<commit_message>
Update example_notebook.ipynb and fake_emdat_test.xlsx to include the new 'GADM Admin Units' column
</commit_message>
<xml_diff>
--- a/data/fake_emdat_test.xlsx
+++ b/data/fake_emdat_test.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20413"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20417"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CEE1AA43-1503-4ED6-95A9-6BB43AC08AD9}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7287FC0-6F6F-446A-900D-B567D3658030}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="38400" windowHeight="17505" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -12,14 +12,14 @@
     <sheet name="EM-DAT Info" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'EM-DAT Data'!$A$1:$AT$101</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'EM-DAT Data'!$A$1:$AU$101</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3679" uniqueCount="626">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3661" uniqueCount="627">
   <si>
     <t>Source:</t>
   </si>
@@ -1897,6 +1897,9 @@
   </si>
   <si>
     <t>[{"adm2_code":198888,"adm2_name":"Honolulu"}]</t>
+  </si>
+  <si>
+    <t>GADM Admin Units</t>
   </si>
 </sst>
 </file>
@@ -2223,7 +2226,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AT101"/>
+  <dimension ref="A1:AU101"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18.140625" customWidth="1"/>
@@ -2243,10 +2246,10 @@
     <col min="18" max="18" width="13.5703125" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="17.7109375" bestFit="1" customWidth="1"/>
     <col min="22" max="22" width="18.7109375" bestFit="1" customWidth="1"/>
-    <col min="44" max="44" width="28.7109375" customWidth="1"/>
+    <col min="44" max="45" width="28.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>13</v>
       </c>
@@ -2380,13 +2383,16 @@
         <v>56</v>
       </c>
       <c r="AS1" t="s">
+        <v>626</v>
+      </c>
+      <c r="AT1" t="s">
         <v>57</v>
       </c>
-      <c r="AT1" t="s">
+      <c r="AU1" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="2" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>604</v>
       </c>
@@ -2519,14 +2525,14 @@
       <c r="AR2" t="s">
         <v>65</v>
       </c>
-      <c r="AS2" t="s">
+      <c r="AT2" t="s">
         <v>386</v>
       </c>
-      <c r="AT2" t="s">
+      <c r="AU2" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="3" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>372</v>
       </c>
@@ -2659,14 +2665,14 @@
       <c r="AR3" t="s">
         <v>65</v>
       </c>
-      <c r="AS3" t="s">
+      <c r="AT3" t="s">
         <v>75</v>
       </c>
-      <c r="AT3" t="s">
+      <c r="AU3" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="4" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>213</v>
       </c>
@@ -2799,14 +2805,14 @@
       <c r="AR4" t="s">
         <v>65</v>
       </c>
-      <c r="AS4" t="s">
+      <c r="AT4" t="s">
         <v>215</v>
       </c>
-      <c r="AT4" t="s">
+      <c r="AU4" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="5" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>559</v>
       </c>
@@ -2939,14 +2945,14 @@
       <c r="AR5" t="s">
         <v>562</v>
       </c>
-      <c r="AS5" t="s">
+      <c r="AT5" t="s">
         <v>558</v>
       </c>
-      <c r="AT5" t="s">
+      <c r="AU5" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="6" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>459</v>
       </c>
@@ -3079,14 +3085,14 @@
       <c r="AR6" t="s">
         <v>65</v>
       </c>
-      <c r="AS6" t="s">
+      <c r="AT6" t="s">
         <v>455</v>
       </c>
-      <c r="AT6" t="s">
+      <c r="AU6" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="7" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>340</v>
       </c>
@@ -3219,14 +3225,14 @@
       <c r="AR7" t="s">
         <v>65</v>
       </c>
-      <c r="AS7" t="s">
+      <c r="AT7" t="s">
         <v>75</v>
       </c>
-      <c r="AT7" t="s">
+      <c r="AU7" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="8" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>375</v>
       </c>
@@ -3359,14 +3365,14 @@
       <c r="AR8" t="s">
         <v>65</v>
       </c>
-      <c r="AS8" t="s">
+      <c r="AT8" t="s">
         <v>75</v>
       </c>
-      <c r="AT8" t="s">
+      <c r="AU8" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="9" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>422</v>
       </c>
@@ -3496,14 +3502,14 @@
       <c r="AQ9">
         <v>59.033144078614221</v>
       </c>
-      <c r="AS9" t="s">
+      <c r="AT9" t="s">
         <v>75</v>
       </c>
-      <c r="AT9" t="s">
+      <c r="AU9" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="10" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>500</v>
       </c>
@@ -3636,14 +3642,14 @@
       <c r="AR10" t="s">
         <v>65</v>
       </c>
-      <c r="AS10" t="s">
+      <c r="AT10" t="s">
         <v>499</v>
       </c>
-      <c r="AT10" t="s">
+      <c r="AU10" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="11" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>357</v>
       </c>
@@ -3776,14 +3782,14 @@
       <c r="AR11" t="s">
         <v>65</v>
       </c>
-      <c r="AS11" t="s">
+      <c r="AT11" t="s">
         <v>75</v>
       </c>
-      <c r="AT11" t="s">
+      <c r="AU11" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="12" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>442</v>
       </c>
@@ -3916,14 +3922,14 @@
       <c r="AR12" t="s">
         <v>65</v>
       </c>
-      <c r="AS12" t="s">
+      <c r="AT12" t="s">
         <v>345</v>
       </c>
-      <c r="AT12" t="s">
+      <c r="AU12" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="13" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>623</v>
       </c>
@@ -4056,14 +4062,14 @@
       <c r="AR13" t="s">
         <v>65</v>
       </c>
-      <c r="AS13" t="s">
+      <c r="AT13" t="s">
         <v>215</v>
       </c>
-      <c r="AT13" t="s">
+      <c r="AU13" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="14" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>556</v>
       </c>
@@ -4196,14 +4202,14 @@
       <c r="AR14" t="s">
         <v>412</v>
       </c>
-      <c r="AS14" t="s">
+      <c r="AT14" t="s">
         <v>554</v>
       </c>
-      <c r="AT14" t="s">
+      <c r="AU14" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="15" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>533</v>
       </c>
@@ -4336,14 +4342,14 @@
       <c r="AR15" t="s">
         <v>535</v>
       </c>
-      <c r="AS15" t="s">
+      <c r="AT15" t="s">
         <v>536</v>
       </c>
-      <c r="AT15" t="s">
+      <c r="AU15" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="16" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>448</v>
       </c>
@@ -4476,14 +4482,14 @@
       <c r="AR16" t="s">
         <v>65</v>
       </c>
-      <c r="AS16" t="s">
+      <c r="AT16" t="s">
         <v>447</v>
       </c>
-      <c r="AT16" t="s">
+      <c r="AU16" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="17" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>583</v>
       </c>
@@ -4616,14 +4622,14 @@
       <c r="AR17" t="s">
         <v>585</v>
       </c>
-      <c r="AS17" t="s">
+      <c r="AT17" t="s">
         <v>582</v>
       </c>
-      <c r="AT17" t="s">
+      <c r="AU17" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="18" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>476</v>
       </c>
@@ -4756,14 +4762,14 @@
       <c r="AR18" t="s">
         <v>65</v>
       </c>
-      <c r="AS18" t="s">
+      <c r="AT18" t="s">
         <v>475</v>
       </c>
-      <c r="AT18" t="s">
+      <c r="AU18" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="19" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>381</v>
       </c>
@@ -4896,14 +4902,14 @@
       <c r="AR19" t="s">
         <v>65</v>
       </c>
-      <c r="AS19" t="s">
+      <c r="AT19" t="s">
         <v>382</v>
       </c>
-      <c r="AT19" t="s">
+      <c r="AU19" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="20" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>373</v>
       </c>
@@ -5036,14 +5042,14 @@
       <c r="AR20" t="s">
         <v>65</v>
       </c>
-      <c r="AS20" t="s">
+      <c r="AT20" t="s">
         <v>75</v>
       </c>
-      <c r="AT20" t="s">
+      <c r="AU20" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="21" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>547</v>
       </c>
@@ -5176,14 +5182,14 @@
       <c r="AR21" t="s">
         <v>65</v>
       </c>
-      <c r="AS21" t="s">
+      <c r="AT21" t="s">
         <v>548</v>
       </c>
-      <c r="AT21" t="s">
+      <c r="AU21" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="22" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>592</v>
       </c>
@@ -5316,14 +5322,14 @@
       <c r="AR22" t="s">
         <v>595</v>
       </c>
-      <c r="AS22" t="s">
+      <c r="AT22" t="s">
         <v>591</v>
       </c>
-      <c r="AT22" t="s">
+      <c r="AU22" t="s">
         <v>590</v>
       </c>
     </row>
-    <row r="23" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>483</v>
       </c>
@@ -5456,14 +5462,14 @@
       <c r="AR23" t="s">
         <v>421</v>
       </c>
-      <c r="AS23" t="s">
+      <c r="AT23" t="s">
         <v>463</v>
       </c>
-      <c r="AT23" t="s">
+      <c r="AU23" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="24" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>567</v>
       </c>
@@ -5596,14 +5602,14 @@
       <c r="AR24" t="s">
         <v>454</v>
       </c>
-      <c r="AS24" t="s">
+      <c r="AT24" t="s">
         <v>566</v>
       </c>
-      <c r="AT24" t="s">
+      <c r="AU24" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="25" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>317</v>
       </c>
@@ -5736,14 +5742,14 @@
       <c r="AR25" t="s">
         <v>65</v>
       </c>
-      <c r="AS25" t="s">
+      <c r="AT25" t="s">
         <v>75</v>
       </c>
-      <c r="AT25" t="s">
+      <c r="AU25" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="26" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>426</v>
       </c>
@@ -5876,14 +5882,14 @@
       <c r="AR26" t="s">
         <v>429</v>
       </c>
-      <c r="AS26" t="s">
+      <c r="AT26" t="s">
         <v>405</v>
       </c>
-      <c r="AT26" t="s">
+      <c r="AU26" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="27" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>310</v>
       </c>
@@ -6016,14 +6022,14 @@
       <c r="AR27" t="s">
         <v>65</v>
       </c>
-      <c r="AS27" t="s">
+      <c r="AT27" t="s">
         <v>75</v>
       </c>
-      <c r="AT27" t="s">
+      <c r="AU27" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="28" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>399</v>
       </c>
@@ -6156,14 +6162,14 @@
       <c r="AR28" t="s">
         <v>65</v>
       </c>
-      <c r="AS28" t="s">
+      <c r="AT28" t="s">
         <v>390</v>
       </c>
-      <c r="AT28" t="s">
+      <c r="AU28" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="29" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>352</v>
       </c>
@@ -6296,14 +6302,14 @@
       <c r="AR29" t="s">
         <v>65</v>
       </c>
-      <c r="AS29" t="s">
+      <c r="AT29" t="s">
         <v>75</v>
       </c>
-      <c r="AT29" t="s">
+      <c r="AU29" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="30" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>509</v>
       </c>
@@ -6436,14 +6442,14 @@
       <c r="AR30" t="s">
         <v>512</v>
       </c>
-      <c r="AS30" t="s">
+      <c r="AT30" t="s">
         <v>507</v>
       </c>
-      <c r="AT30" t="s">
+      <c r="AU30" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="31" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>450</v>
       </c>
@@ -6576,14 +6582,14 @@
       <c r="AR31" t="s">
         <v>414</v>
       </c>
-      <c r="AS31" t="s">
+      <c r="AT31" t="s">
         <v>446</v>
       </c>
-      <c r="AT31" t="s">
+      <c r="AU31" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="32" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>320</v>
       </c>
@@ -6716,14 +6722,14 @@
       <c r="AR32" t="s">
         <v>65</v>
       </c>
-      <c r="AS32" t="s">
+      <c r="AT32" t="s">
         <v>75</v>
       </c>
-      <c r="AT32" t="s">
+      <c r="AU32" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="33" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>505</v>
       </c>
@@ -6853,14 +6859,14 @@
       <c r="AR33" t="s">
         <v>65</v>
       </c>
-      <c r="AS33" t="s">
+      <c r="AT33" t="s">
         <v>398</v>
       </c>
-      <c r="AT33" t="s">
+      <c r="AU33" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="34" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>522</v>
       </c>
@@ -6993,14 +6999,14 @@
       <c r="AR34" t="s">
         <v>525</v>
       </c>
-      <c r="AS34" t="s">
+      <c r="AT34" t="s">
         <v>521</v>
       </c>
-      <c r="AT34" t="s">
+      <c r="AU34" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="35" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>350</v>
       </c>
@@ -7133,14 +7139,14 @@
       <c r="AR35" t="s">
         <v>65</v>
       </c>
-      <c r="AS35" t="s">
+      <c r="AT35" t="s">
         <v>75</v>
       </c>
-      <c r="AT35" t="s">
+      <c r="AU35" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="36" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>486</v>
       </c>
@@ -7273,14 +7279,14 @@
       <c r="AR36" t="s">
         <v>65</v>
       </c>
-      <c r="AS36" t="s">
+      <c r="AT36" t="s">
         <v>485</v>
       </c>
-      <c r="AT36" t="s">
+      <c r="AU36" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="37" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>303</v>
       </c>
@@ -7413,14 +7419,14 @@
       <c r="AR37" t="s">
         <v>65</v>
       </c>
-      <c r="AS37" t="s">
+      <c r="AT37" t="s">
         <v>293</v>
       </c>
-      <c r="AT37" t="s">
+      <c r="AU37" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="38" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>360</v>
       </c>
@@ -7553,14 +7559,14 @@
       <c r="AR38" t="s">
         <v>65</v>
       </c>
-      <c r="AS38" t="s">
+      <c r="AT38" t="s">
         <v>75</v>
       </c>
-      <c r="AT38" t="s">
+      <c r="AU38" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="39" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>461</v>
       </c>
@@ -7693,14 +7699,14 @@
       <c r="AR39" t="s">
         <v>65</v>
       </c>
-      <c r="AS39" t="s">
+      <c r="AT39" t="s">
         <v>364</v>
       </c>
-      <c r="AT39" t="s">
+      <c r="AU39" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="40" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>490</v>
       </c>
@@ -7833,14 +7839,14 @@
       <c r="AR40" t="s">
         <v>65</v>
       </c>
-      <c r="AS40" t="s">
+      <c r="AT40" t="s">
         <v>321</v>
       </c>
-      <c r="AT40" t="s">
+      <c r="AU40" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="41" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>306</v>
       </c>
@@ -7973,14 +7979,14 @@
       <c r="AR41" t="s">
         <v>65</v>
       </c>
-      <c r="AS41" t="s">
+      <c r="AT41" t="s">
         <v>130</v>
       </c>
-      <c r="AT41" t="s">
+      <c r="AU41" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="42" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>402</v>
       </c>
@@ -8113,14 +8119,15 @@
       <c r="AR42" s="1" t="s">
         <v>620</v>
       </c>
-      <c r="AS42" t="s">
+      <c r="AS42" s="1"/>
+      <c r="AT42" t="s">
         <v>75</v>
       </c>
-      <c r="AT42" t="s">
+      <c r="AU42" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="43" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>497</v>
       </c>
@@ -8253,14 +8260,14 @@
       <c r="AR43" t="s">
         <v>493</v>
       </c>
-      <c r="AS43" s="2" t="s">
+      <c r="AT43" s="2" t="s">
         <v>621</v>
       </c>
-      <c r="AT43" t="s">
+      <c r="AU43" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="44" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>376</v>
       </c>
@@ -8393,14 +8400,14 @@
       <c r="AR44" t="s">
         <v>65</v>
       </c>
-      <c r="AS44" t="s">
+      <c r="AT44" t="s">
         <v>75</v>
       </c>
-      <c r="AT44" s="2" t="s">
+      <c r="AU44" s="2" t="s">
         <v>622</v>
       </c>
     </row>
-    <row r="45" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>513</v>
       </c>
@@ -8531,14 +8538,14 @@
       <c r="AR45" t="s">
         <v>516</v>
       </c>
-      <c r="AS45" t="s">
+      <c r="AT45" t="s">
         <v>508</v>
       </c>
-      <c r="AT45" t="s">
+      <c r="AU45" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="46" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>529</v>
       </c>
@@ -8669,14 +8676,14 @@
       <c r="AR46" t="s">
         <v>531</v>
       </c>
-      <c r="AS46" t="s">
+      <c r="AT46" t="s">
         <v>528</v>
       </c>
-      <c r="AT46" t="s">
+      <c r="AU46" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="47" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>579</v>
       </c>
@@ -8809,14 +8816,14 @@
       <c r="AR47" t="s">
         <v>581</v>
       </c>
-      <c r="AS47" t="s">
+      <c r="AT47" t="s">
         <v>569</v>
       </c>
-      <c r="AT47" t="s">
+      <c r="AU47" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="48" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>564</v>
       </c>
@@ -8949,14 +8956,14 @@
       <c r="AR48" t="s">
         <v>65</v>
       </c>
-      <c r="AS48" t="s">
+      <c r="AT48" t="s">
         <v>563</v>
       </c>
-      <c r="AT48" t="s">
+      <c r="AU48" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="49" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>546</v>
       </c>
@@ -9089,14 +9096,14 @@
       <c r="AR49" t="s">
         <v>65</v>
       </c>
-      <c r="AS49" t="s">
+      <c r="AT49" t="s">
         <v>545</v>
       </c>
-      <c r="AT49" t="s">
+      <c r="AU49" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="50" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>437</v>
       </c>
@@ -9229,14 +9236,14 @@
       <c r="AR50" t="s">
         <v>439</v>
       </c>
-      <c r="AS50" t="s">
+      <c r="AT50" t="s">
         <v>115</v>
       </c>
-      <c r="AT50" t="s">
+      <c r="AU50" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="51" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>441</v>
       </c>
@@ -9369,14 +9376,14 @@
       <c r="AR51" t="s">
         <v>65</v>
       </c>
-      <c r="AS51" t="s">
+      <c r="AT51" t="s">
         <v>440</v>
       </c>
-      <c r="AT51" t="s">
+      <c r="AU51" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="52" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>527</v>
       </c>
@@ -9509,14 +9516,14 @@
       <c r="AR52" t="s">
         <v>457</v>
       </c>
-      <c r="AS52" t="s">
+      <c r="AT52" t="s">
         <v>526</v>
       </c>
-      <c r="AT52" t="s">
+      <c r="AU52" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="53" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>316</v>
       </c>
@@ -9649,14 +9656,14 @@
       <c r="AR53" t="s">
         <v>65</v>
       </c>
-      <c r="AS53" t="s">
+      <c r="AT53" t="s">
         <v>75</v>
       </c>
-      <c r="AT53" t="s">
+      <c r="AU53" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="54" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>538</v>
       </c>
@@ -9789,14 +9796,14 @@
       <c r="AR54" t="s">
         <v>494</v>
       </c>
-      <c r="AS54" t="s">
+      <c r="AT54" t="s">
         <v>537</v>
       </c>
-      <c r="AT54" t="s">
+      <c r="AU54" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="55" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>596</v>
       </c>
@@ -9929,14 +9936,14 @@
       <c r="AR55" t="s">
         <v>65</v>
       </c>
-      <c r="AS55" t="s">
+      <c r="AT55" t="s">
         <v>599</v>
       </c>
-      <c r="AT55" t="s">
+      <c r="AU55" t="s">
         <v>590</v>
       </c>
     </row>
-    <row r="56" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>296</v>
       </c>
@@ -10069,14 +10076,14 @@
       <c r="AR56" t="s">
         <v>65</v>
       </c>
-      <c r="AS56" t="s">
+      <c r="AT56" t="s">
         <v>286</v>
       </c>
-      <c r="AT56" t="s">
+      <c r="AU56" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="57" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>403</v>
       </c>
@@ -10209,14 +10216,14 @@
       <c r="AR57" t="s">
         <v>65</v>
       </c>
-      <c r="AS57" t="s">
+      <c r="AT57" t="s">
         <v>75</v>
       </c>
-      <c r="AT57" t="s">
+      <c r="AU57" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="58" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>464</v>
       </c>
@@ -10349,14 +10356,14 @@
       <c r="AR58" t="s">
         <v>466</v>
       </c>
-      <c r="AS58" t="s">
+      <c r="AT58" t="s">
         <v>467</v>
       </c>
-      <c r="AT58" t="s">
+      <c r="AU58" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="59" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>270</v>
       </c>
@@ -10489,14 +10496,14 @@
       <c r="AR59" t="s">
         <v>65</v>
       </c>
-      <c r="AS59" t="s">
+      <c r="AT59" t="s">
         <v>75</v>
       </c>
-      <c r="AT59" t="s">
+      <c r="AU59" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="60" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>415</v>
       </c>
@@ -10629,14 +10636,14 @@
       <c r="AR60" t="s">
         <v>65</v>
       </c>
-      <c r="AS60" t="s">
+      <c r="AT60" t="s">
         <v>75</v>
       </c>
-      <c r="AT60" t="s">
+      <c r="AU60" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="61" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>452</v>
       </c>
@@ -10769,14 +10776,15 @@
       <c r="AR61" s="1" t="s">
         <v>625</v>
       </c>
-      <c r="AS61" t="s">
+      <c r="AS61" s="1"/>
+      <c r="AT61" t="s">
         <v>451</v>
       </c>
-      <c r="AT61" t="s">
+      <c r="AU61" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="62" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>204</v>
       </c>
@@ -10909,14 +10917,14 @@
       <c r="AR62" t="s">
         <v>65</v>
       </c>
-      <c r="AS62" t="s">
+      <c r="AT62" t="s">
         <v>75</v>
       </c>
-      <c r="AT62" t="s">
+      <c r="AU62" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="63" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>586</v>
       </c>
@@ -11049,14 +11057,14 @@
       <c r="AR63" t="s">
         <v>588</v>
       </c>
-      <c r="AS63" t="s">
+      <c r="AT63" t="s">
         <v>589</v>
       </c>
-      <c r="AT63" t="s">
+      <c r="AU63" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="64" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>311</v>
       </c>
@@ -11189,14 +11197,14 @@
       <c r="AR64" t="s">
         <v>65</v>
       </c>
-      <c r="AS64" t="s">
+      <c r="AT64" t="s">
         <v>75</v>
       </c>
-      <c r="AT64" t="s">
+      <c r="AU64" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="65" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>392</v>
       </c>
@@ -11329,14 +11337,14 @@
       <c r="AR65" t="s">
         <v>65</v>
       </c>
-      <c r="AS65" t="s">
+      <c r="AT65" t="s">
         <v>75</v>
       </c>
-      <c r="AT65" t="s">
+      <c r="AU65" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="66" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>333</v>
       </c>
@@ -11469,14 +11477,14 @@
       <c r="AR66" t="s">
         <v>65</v>
       </c>
-      <c r="AS66" t="s">
+      <c r="AT66" t="s">
         <v>75</v>
       </c>
-      <c r="AT66" t="s">
+      <c r="AU66" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="67" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>430</v>
       </c>
@@ -11609,14 +11617,14 @@
       <c r="AR67" t="s">
         <v>65</v>
       </c>
-      <c r="AS67" t="s">
+      <c r="AT67" t="s">
         <v>75</v>
       </c>
-      <c r="AT67" t="s">
+      <c r="AU67" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="68" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>287</v>
       </c>
@@ -11749,14 +11757,14 @@
       <c r="AR68" t="s">
         <v>65</v>
       </c>
-      <c r="AS68" t="s">
+      <c r="AT68" t="s">
         <v>75</v>
       </c>
-      <c r="AT68" t="s">
+      <c r="AU68" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="69" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>378</v>
       </c>
@@ -11889,14 +11897,14 @@
       <c r="AR69" t="s">
         <v>65</v>
       </c>
-      <c r="AS69" t="s">
+      <c r="AT69" t="s">
         <v>75</v>
       </c>
-      <c r="AT69" t="s">
+      <c r="AU69" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="70" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>424</v>
       </c>
@@ -12029,14 +12037,15 @@
       <c r="AR70" s="1" t="s">
         <v>624</v>
       </c>
-      <c r="AS70" t="s">
+      <c r="AS70" s="1"/>
+      <c r="AT70" t="s">
         <v>75</v>
       </c>
-      <c r="AT70" t="s">
+      <c r="AU70" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="71" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>338</v>
       </c>
@@ -12169,14 +12178,14 @@
       <c r="AR71" t="s">
         <v>65</v>
       </c>
-      <c r="AS71" t="s">
+      <c r="AT71" t="s">
         <v>75</v>
       </c>
-      <c r="AT71" t="s">
+      <c r="AU71" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="72" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>419</v>
       </c>
@@ -12309,14 +12318,14 @@
       <c r="AR72" t="s">
         <v>65</v>
       </c>
-      <c r="AS72" t="s">
+      <c r="AT72" t="s">
         <v>401</v>
       </c>
-      <c r="AT72" t="s">
+      <c r="AU72" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="73" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>394</v>
       </c>
@@ -12449,14 +12458,14 @@
       <c r="AR73" t="s">
         <v>65</v>
       </c>
-      <c r="AS73" t="s">
+      <c r="AT73" t="s">
         <v>75</v>
       </c>
-      <c r="AT73" t="s">
+      <c r="AU73" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="74" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>571</v>
       </c>
@@ -12589,14 +12598,14 @@
       <c r="AR74" t="s">
         <v>65</v>
       </c>
-      <c r="AS74" t="s">
+      <c r="AT74" t="s">
         <v>570</v>
       </c>
-      <c r="AT74" t="s">
+      <c r="AU74" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="75" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>347</v>
       </c>
@@ -12729,14 +12738,14 @@
       <c r="AR75" t="s">
         <v>65</v>
       </c>
-      <c r="AS75" t="s">
+      <c r="AT75" t="s">
         <v>346</v>
       </c>
-      <c r="AT75" t="s">
+      <c r="AU75" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="76" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>206</v>
       </c>
@@ -12869,14 +12878,14 @@
       <c r="AR76" t="s">
         <v>65</v>
       </c>
-      <c r="AS76" t="s">
+      <c r="AT76" t="s">
         <v>208</v>
       </c>
-      <c r="AT76" t="s">
+      <c r="AU76" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="77" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>444</v>
       </c>
@@ -13009,14 +13018,14 @@
       <c r="AR77" t="s">
         <v>65</v>
       </c>
-      <c r="AS77" t="s">
+      <c r="AT77" t="s">
         <v>328</v>
       </c>
-      <c r="AT77" t="s">
+      <c r="AU77" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="78" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>226</v>
       </c>
@@ -13149,14 +13158,14 @@
       <c r="AR78" t="s">
         <v>65</v>
       </c>
-      <c r="AS78" t="s">
+      <c r="AT78" t="s">
         <v>225</v>
       </c>
-      <c r="AT78" t="s">
+      <c r="AU78" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="79" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>344</v>
       </c>
@@ -13289,14 +13298,14 @@
       <c r="AR79" t="s">
         <v>65</v>
       </c>
-      <c r="AS79" t="s">
+      <c r="AT79" t="s">
         <v>75</v>
       </c>
-      <c r="AT79" t="s">
+      <c r="AU79" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="80" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>489</v>
       </c>
@@ -13429,14 +13438,14 @@
       <c r="AR80" t="s">
         <v>65</v>
       </c>
-      <c r="AS80" t="s">
+      <c r="AT80" t="s">
         <v>488</v>
       </c>
-      <c r="AT80" t="s">
+      <c r="AU80" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="81" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>577</v>
       </c>
@@ -13569,14 +13578,14 @@
       <c r="AR81" t="s">
         <v>65</v>
       </c>
-      <c r="AS81" t="s">
+      <c r="AT81" t="s">
         <v>576</v>
       </c>
-      <c r="AT81" t="s">
+      <c r="AU81" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="82" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>294</v>
       </c>
@@ -13709,14 +13718,14 @@
       <c r="AR82" t="s">
         <v>65</v>
       </c>
-      <c r="AS82" t="s">
+      <c r="AT82" t="s">
         <v>239</v>
       </c>
-      <c r="AT82" t="s">
+      <c r="AU82" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="83" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>331</v>
       </c>
@@ -13849,14 +13858,14 @@
       <c r="AR83" t="s">
         <v>65</v>
       </c>
-      <c r="AS83" t="s">
+      <c r="AT83" t="s">
         <v>75</v>
       </c>
-      <c r="AT83" t="s">
+      <c r="AU83" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="84" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>406</v>
       </c>
@@ -13989,14 +13998,14 @@
       <c r="AR84" t="s">
         <v>408</v>
       </c>
-      <c r="AS84" t="s">
+      <c r="AT84" t="s">
         <v>75</v>
       </c>
-      <c r="AT84" t="s">
+      <c r="AU84" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="85" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>304</v>
       </c>
@@ -14129,14 +14138,14 @@
       <c r="AR85" t="s">
         <v>65</v>
       </c>
-      <c r="AS85" t="s">
+      <c r="AT85" t="s">
         <v>297</v>
       </c>
-      <c r="AT85" t="s">
+      <c r="AU85" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="86" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
         <v>417</v>
       </c>
@@ -14269,14 +14278,14 @@
       <c r="AR86" t="s">
         <v>65</v>
       </c>
-      <c r="AS86" t="s">
+      <c r="AT86" t="s">
         <v>75</v>
       </c>
-      <c r="AT86" t="s">
+      <c r="AU86" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="87" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
         <v>479</v>
       </c>
@@ -14409,14 +14418,14 @@
       <c r="AR87" t="s">
         <v>65</v>
       </c>
-      <c r="AS87" t="s">
+      <c r="AT87" t="s">
         <v>469</v>
       </c>
-      <c r="AT87" t="s">
+      <c r="AU87" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="88" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
         <v>495</v>
       </c>
@@ -14549,14 +14558,14 @@
       <c r="AR88" t="s">
         <v>432</v>
       </c>
-      <c r="AS88" t="s">
+      <c r="AT88" t="s">
         <v>492</v>
       </c>
-      <c r="AT88" t="s">
+      <c r="AU88" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="89" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
         <v>503</v>
       </c>
@@ -14687,14 +14696,14 @@
       <c r="AR89" t="s">
         <v>65</v>
       </c>
-      <c r="AS89" t="s">
+      <c r="AT89" t="s">
         <v>502</v>
       </c>
-      <c r="AT89" t="s">
+      <c r="AU89" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="90" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
         <v>354</v>
       </c>
@@ -14824,14 +14833,14 @@
       <c r="AR90" t="s">
         <v>65</v>
       </c>
-      <c r="AS90" t="s">
+      <c r="AT90" t="s">
         <v>337</v>
       </c>
-      <c r="AT90" t="s">
+      <c r="AU90" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="91" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
         <v>602</v>
       </c>
@@ -14964,14 +14973,14 @@
       <c r="AR91" t="s">
         <v>65</v>
       </c>
-      <c r="AS91" t="s">
+      <c r="AT91" t="s">
         <v>600</v>
       </c>
-      <c r="AT91" t="s">
+      <c r="AU91" t="s">
         <v>601</v>
       </c>
     </row>
-    <row r="92" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
         <v>324</v>
       </c>
@@ -15104,14 +15113,14 @@
       <c r="AR92" t="s">
         <v>65</v>
       </c>
-      <c r="AS92" t="s">
+      <c r="AT92" t="s">
         <v>326</v>
       </c>
-      <c r="AT92" t="s">
+      <c r="AU92" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="93" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
         <v>470</v>
       </c>
@@ -15244,14 +15253,14 @@
       <c r="AR93" t="s">
         <v>474</v>
       </c>
-      <c r="AS93" t="s">
+      <c r="AT93" t="s">
         <v>468</v>
       </c>
-      <c r="AT93" t="s">
+      <c r="AU93" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="94" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
         <v>550</v>
       </c>
@@ -15384,14 +15393,14 @@
       <c r="AR94" t="s">
         <v>552</v>
       </c>
-      <c r="AS94" t="s">
+      <c r="AT94" t="s">
         <v>553</v>
       </c>
-      <c r="AT94" t="s">
+      <c r="AU94" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="95" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
         <v>517</v>
       </c>
@@ -15524,14 +15533,14 @@
       <c r="AR95" t="s">
         <v>411</v>
       </c>
-      <c r="AS95" t="s">
+      <c r="AT95" t="s">
         <v>520</v>
       </c>
-      <c r="AT95" t="s">
+      <c r="AU95" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="96" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
         <v>541</v>
       </c>
@@ -15664,14 +15673,14 @@
       <c r="AR96" t="s">
         <v>65</v>
       </c>
-      <c r="AS96" t="s">
+      <c r="AT96" t="s">
         <v>544</v>
       </c>
-      <c r="AT96" t="s">
+      <c r="AU96" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="97" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
         <v>573</v>
       </c>
@@ -15804,14 +15813,14 @@
       <c r="AR97" t="s">
         <v>575</v>
       </c>
-      <c r="AS97" t="s">
+      <c r="AT97" t="s">
         <v>572</v>
       </c>
-      <c r="AT97" t="s">
+      <c r="AU97" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="98" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
         <v>309</v>
       </c>
@@ -15944,14 +15953,14 @@
       <c r="AR98" t="s">
         <v>65</v>
       </c>
-      <c r="AS98" t="s">
+      <c r="AT98" t="s">
         <v>75</v>
       </c>
-      <c r="AT98" t="s">
+      <c r="AU98" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="99" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
         <v>433</v>
       </c>
@@ -16084,14 +16093,14 @@
       <c r="AR99" t="s">
         <v>436</v>
       </c>
-      <c r="AS99" t="s">
+      <c r="AT99" t="s">
         <v>308</v>
       </c>
-      <c r="AT99" t="s">
+      <c r="AU99" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="100" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
         <v>322</v>
       </c>
@@ -16224,14 +16233,14 @@
       <c r="AR100" t="s">
         <v>65</v>
       </c>
-      <c r="AS100" t="s">
+      <c r="AT100" t="s">
         <v>75</v>
       </c>
-      <c r="AT100" t="s">
+      <c r="AU100" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="101" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
         <v>370</v>
       </c>
@@ -16364,16 +16373,16 @@
       <c r="AR101" t="s">
         <v>65</v>
       </c>
-      <c r="AS101" t="s">
+      <c r="AT101" t="s">
         <v>369</v>
       </c>
-      <c r="AT101" t="s">
+      <c r="AU101" t="s">
         <v>76</v>
       </c>
     </row>
   </sheetData>
-  <sortState ref="A5:AU26737">
-    <sortCondition ref="AU1"/>
+  <sortState ref="A5:AV26737">
+    <sortCondition ref="AV1"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>